<commit_message>
Add 2-week colspan handling in weekly view
Introduce planRow callback to compute per-row week spans (colspan=1|2) based on cardDurations and técnica assignments, using a consumed set to skip the next week when a span-2 occurs. Update the table rendering to iterate over planRow results and set <td colSpan={span}>, so activities or labels with duration=2 render across two weeks. Also update the planeacion spreadsheet (docs/planeacion_semanal/PLANEACION SEMANAL GRD.xlsx). This enables proper rendering of multi-week cards in PlaneacionSemanalView.
</commit_message>
<xml_diff>
--- a/docs/planeacion_semanal/PLANEACION SEMANAL GRD.xlsx
+++ b/docs/planeacion_semanal/PLANEACION SEMANAL GRD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David\Documents\GitHub\asistencia-sena\docs\planeacion_semanal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC48FF1E-BBF7-4BFE-847D-CE6664D7320C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5C92CD-5EC1-4B07-9AFB-186C88F3B279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12480" xr2:uid="{6CA533EF-C929-4BFD-B5C5-4031C7FF55EC}"/>
   </bookViews>
@@ -2847,7 +2847,7 @@
     <col min="121" max="121" width="18.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:121" ht="17.399999999999999" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:121" ht="10.8" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2970,7 +2970,7 @@
       <c r="DP1" s="8"/>
       <c r="DQ1" s="8"/>
     </row>
-    <row r="2" spans="1:121" ht="45" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:121" ht="30.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="9" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
Add per-week date overrides to weekly plan
Allow anchoring/overriding the start date for individual weeks in the Planeacion Semanal UI and persist the data. Changes include:

- types.ts: add weekDateOverrides to PlaneacionSemanalFichaData (weekIndex → ISO date).
- services/db.ts: merge weekDateOverrides when combining local/cloud records.
- views/PlaneacionSemanalView.tsx: implement buildWeekDates to compute week starts/ends from a base date and apply overrides; add UI to open a datepicker per-week, set/clear overrides, persist changes, and recompute displayed dates; small UX tweaks (close picker on grid click, auto-show picker focus).
- Updated planning spreadsheet binary (docs/planeacion_semanal/PLANEACION SEMANAL GRD.xlsx).

This enables shifting a given week's start date and recalculates subsequent weeks accordingly, useful for schedule corrections without changing the global base date.
</commit_message>
<xml_diff>
--- a/docs/planeacion_semanal/PLANEACION SEMANAL GRD.xlsx
+++ b/docs/planeacion_semanal/PLANEACION SEMANAL GRD.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David\Documents\GitHub\asistencia-sena\docs\planeacion_semanal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5C92CD-5EC1-4B07-9AFB-186C88F3B279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9462A22-2D82-43CC-9B1A-5115E087FCA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12480" xr2:uid="{6CA533EF-C929-4BFD-B5C5-4031C7FF55EC}"/>
   </bookViews>
@@ -3661,417 +3661,416 @@
         <v>45999</v>
       </c>
       <c r="N5" s="53">
-        <f>M5+7</f>
-        <v>46006</v>
+        <v>46055</v>
       </c>
       <c r="O5" s="57" t="s">
         <v>40</v>
       </c>
       <c r="P5" s="55">
         <f>N5+7</f>
-        <v>46013</v>
+        <v>46062</v>
       </c>
       <c r="Q5" s="56">
         <f>P5+7</f>
-        <v>46020</v>
+        <v>46069</v>
       </c>
       <c r="R5" s="56">
         <f>Q5+7</f>
-        <v>46027</v>
+        <v>46076</v>
       </c>
       <c r="S5" s="56">
         <f>R5+7</f>
-        <v>46034</v>
+        <v>46083</v>
       </c>
       <c r="T5" s="56">
         <f>S5+7</f>
-        <v>46041</v>
+        <v>46090</v>
       </c>
       <c r="U5" s="56">
         <f>T5+7</f>
-        <v>46048</v>
+        <v>46097</v>
       </c>
       <c r="V5" s="56">
         <f>U5+7</f>
-        <v>46055</v>
+        <v>46104</v>
       </c>
       <c r="W5" s="56">
         <f>V5+7</f>
-        <v>46062</v>
+        <v>46111</v>
       </c>
       <c r="X5" s="56">
         <f>W5+7</f>
-        <v>46069</v>
+        <v>46118</v>
       </c>
       <c r="Y5" s="56">
         <f>X5+7</f>
-        <v>46076</v>
+        <v>46125</v>
       </c>
       <c r="Z5" s="56">
         <f>Y5+7</f>
-        <v>46083</v>
+        <v>46132</v>
       </c>
       <c r="AA5" s="53">
         <f>Z5+7</f>
-        <v>46090</v>
+        <v>46139</v>
       </c>
       <c r="AB5" s="57" t="s">
         <v>40</v>
       </c>
       <c r="AC5" s="55">
         <f>AA5+7</f>
-        <v>46097</v>
+        <v>46146</v>
       </c>
       <c r="AD5" s="56">
         <f>AC5+7</f>
-        <v>46104</v>
+        <v>46153</v>
       </c>
       <c r="AE5" s="56">
         <f>AD5+7</f>
-        <v>46111</v>
+        <v>46160</v>
       </c>
       <c r="AF5" s="56">
         <f>AE5+7</f>
-        <v>46118</v>
+        <v>46167</v>
       </c>
       <c r="AG5" s="56">
         <f>AF5+7</f>
-        <v>46125</v>
+        <v>46174</v>
       </c>
       <c r="AH5" s="56">
         <f>AG5+7</f>
-        <v>46132</v>
+        <v>46181</v>
       </c>
       <c r="AI5" s="56">
         <f>AH5+7</f>
-        <v>46139</v>
+        <v>46188</v>
       </c>
       <c r="AJ5" s="56">
         <f>AI5+7</f>
-        <v>46146</v>
+        <v>46195</v>
       </c>
       <c r="AK5" s="56">
         <f>AJ5+7</f>
-        <v>46153</v>
+        <v>46202</v>
       </c>
       <c r="AL5" s="56">
         <f>AK5+7</f>
-        <v>46160</v>
+        <v>46209</v>
       </c>
       <c r="AM5" s="56">
         <f>AL5+7</f>
-        <v>46167</v>
+        <v>46216</v>
       </c>
       <c r="AN5" s="53">
         <f>AM5+7</f>
-        <v>46174</v>
+        <v>46223</v>
       </c>
       <c r="AO5" s="58" t="s">
         <v>40</v>
       </c>
       <c r="AP5" s="55">
         <f>AN5+7</f>
-        <v>46181</v>
+        <v>46230</v>
       </c>
       <c r="AQ5" s="56">
         <f>AP5+7</f>
-        <v>46188</v>
+        <v>46237</v>
       </c>
       <c r="AR5" s="56">
         <f>AQ5+7</f>
-        <v>46195</v>
+        <v>46244</v>
       </c>
       <c r="AS5" s="56">
         <f>AR5+7</f>
-        <v>46202</v>
+        <v>46251</v>
       </c>
       <c r="AT5" s="56">
         <f>AS5+7</f>
-        <v>46209</v>
+        <v>46258</v>
       </c>
       <c r="AU5" s="56">
         <f>AT5+7</f>
-        <v>46216</v>
+        <v>46265</v>
       </c>
       <c r="AV5" s="56">
         <f>AU5+7</f>
-        <v>46223</v>
+        <v>46272</v>
       </c>
       <c r="AW5" s="56">
         <f>AV5+7</f>
-        <v>46230</v>
+        <v>46279</v>
       </c>
       <c r="AX5" s="56">
         <f>AW5+7</f>
-        <v>46237</v>
+        <v>46286</v>
       </c>
       <c r="AY5" s="56">
         <f>AX5+7</f>
-        <v>46244</v>
+        <v>46293</v>
       </c>
       <c r="AZ5" s="56">
         <f>AY5+7</f>
-        <v>46251</v>
+        <v>46300</v>
       </c>
       <c r="BA5" s="53">
         <f>AZ5+7</f>
-        <v>46258</v>
+        <v>46307</v>
       </c>
       <c r="BB5" s="58" t="s">
         <v>40</v>
       </c>
       <c r="BC5" s="55">
         <f>BA5+7</f>
-        <v>46265</v>
+        <v>46314</v>
       </c>
       <c r="BD5" s="56">
         <f>BC5+7</f>
-        <v>46272</v>
+        <v>46321</v>
       </c>
       <c r="BE5" s="56">
         <f>BD5+7</f>
-        <v>46279</v>
+        <v>46328</v>
       </c>
       <c r="BF5" s="56">
         <f>BE5+7</f>
-        <v>46286</v>
+        <v>46335</v>
       </c>
       <c r="BG5" s="56">
         <f>BF5+7</f>
-        <v>46293</v>
+        <v>46342</v>
       </c>
       <c r="BH5" s="56">
         <f>BG5+7</f>
-        <v>46300</v>
+        <v>46349</v>
       </c>
       <c r="BI5" s="56">
         <f>BH5+7</f>
-        <v>46307</v>
+        <v>46356</v>
       </c>
       <c r="BJ5" s="56">
         <f>BI5+7</f>
-        <v>46314</v>
+        <v>46363</v>
       </c>
       <c r="BK5" s="56">
         <f>BJ5+7</f>
-        <v>46321</v>
+        <v>46370</v>
       </c>
       <c r="BL5" s="56">
         <f>BK5+7</f>
-        <v>46328</v>
+        <v>46377</v>
       </c>
       <c r="BM5" s="56">
         <f>BL5+7</f>
-        <v>46335</v>
+        <v>46384</v>
       </c>
       <c r="BN5" s="53">
         <f>BM5+7</f>
-        <v>46342</v>
+        <v>46391</v>
       </c>
       <c r="BO5" s="58" t="s">
         <v>40</v>
       </c>
       <c r="BP5" s="55">
         <f>BN5+7</f>
-        <v>46349</v>
+        <v>46398</v>
       </c>
       <c r="BQ5" s="56">
         <f>BP5+7</f>
-        <v>46356</v>
+        <v>46405</v>
       </c>
       <c r="BR5" s="56">
         <f>BQ5+7</f>
-        <v>46363</v>
+        <v>46412</v>
       </c>
       <c r="BS5" s="56">
         <f>BR5+7</f>
-        <v>46370</v>
+        <v>46419</v>
       </c>
       <c r="BT5" s="56">
         <f>BS5+7</f>
-        <v>46377</v>
+        <v>46426</v>
       </c>
       <c r="BU5" s="56">
         <f>BT5+7</f>
-        <v>46384</v>
+        <v>46433</v>
       </c>
       <c r="BV5" s="56">
         <f>BU5+7</f>
-        <v>46391</v>
+        <v>46440</v>
       </c>
       <c r="BW5" s="53">
         <f>BV5+7</f>
-        <v>46398</v>
+        <v>46447</v>
       </c>
       <c r="BX5" s="58" t="s">
         <v>40</v>
       </c>
       <c r="BY5" s="55">
         <f>BW5+7</f>
-        <v>46405</v>
+        <v>46454</v>
       </c>
       <c r="BZ5" s="56">
         <f>BY5+7</f>
-        <v>46412</v>
+        <v>46461</v>
       </c>
       <c r="CA5" s="56">
         <f>BZ5+7</f>
-        <v>46419</v>
+        <v>46468</v>
       </c>
       <c r="CB5" s="56">
         <f>CA5+7</f>
-        <v>46426</v>
+        <v>46475</v>
       </c>
       <c r="CC5" s="56">
         <f>CB5+7</f>
-        <v>46433</v>
+        <v>46482</v>
       </c>
       <c r="CD5" s="56">
         <f>CC5+7</f>
-        <v>46440</v>
+        <v>46489</v>
       </c>
       <c r="CE5" s="56">
         <f>CD5+7</f>
-        <v>46447</v>
+        <v>46496</v>
       </c>
       <c r="CF5" s="53">
         <f>CE5+7</f>
-        <v>46454</v>
+        <v>46503</v>
       </c>
       <c r="CG5" s="59" t="s">
         <v>40</v>
       </c>
       <c r="CH5" s="55">
         <f>CF5+7</f>
-        <v>46461</v>
+        <v>46510</v>
       </c>
       <c r="CI5" s="56">
         <f>CH5+7</f>
-        <v>46468</v>
+        <v>46517</v>
       </c>
       <c r="CJ5" s="56">
         <f>CI5+7</f>
-        <v>46475</v>
+        <v>46524</v>
       </c>
       <c r="CK5" s="56">
         <f>CJ5+7</f>
-        <v>46482</v>
+        <v>46531</v>
       </c>
       <c r="CL5" s="56">
         <f>CK5+7</f>
-        <v>46489</v>
+        <v>46538</v>
       </c>
       <c r="CM5" s="56">
         <f>CL5+7</f>
-        <v>46496</v>
+        <v>46545</v>
       </c>
       <c r="CN5" s="56">
         <f>CM5+7</f>
-        <v>46503</v>
+        <v>46552</v>
       </c>
       <c r="CO5" s="53">
         <f>CN5+7</f>
-        <v>46510</v>
+        <v>46559</v>
       </c>
       <c r="CP5" s="59" t="s">
         <v>40</v>
       </c>
       <c r="CQ5" s="55">
         <f>CO5+7</f>
-        <v>46517</v>
+        <v>46566</v>
       </c>
       <c r="CR5" s="56">
         <f>CQ5+7</f>
-        <v>46524</v>
+        <v>46573</v>
       </c>
       <c r="CS5" s="56">
         <f>CR5+7</f>
-        <v>46531</v>
+        <v>46580</v>
       </c>
       <c r="CT5" s="56">
         <f>CS5+7</f>
-        <v>46538</v>
+        <v>46587</v>
       </c>
       <c r="CU5" s="56">
         <f>CT5+7</f>
-        <v>46545</v>
+        <v>46594</v>
       </c>
       <c r="CV5" s="53">
         <f>CU5+7</f>
-        <v>46552</v>
+        <v>46601</v>
       </c>
       <c r="CW5" s="59" t="s">
         <v>40</v>
       </c>
       <c r="CX5" s="55">
         <f>CV5+7</f>
-        <v>46559</v>
+        <v>46608</v>
       </c>
       <c r="CY5" s="56">
         <f>CX5+7</f>
-        <v>46566</v>
+        <v>46615</v>
       </c>
       <c r="CZ5" s="56">
         <f>CY5+7</f>
-        <v>46573</v>
+        <v>46622</v>
       </c>
       <c r="DA5" s="56">
         <f>CZ5+7</f>
-        <v>46580</v>
+        <v>46629</v>
       </c>
       <c r="DB5" s="56">
         <f>DA5+7</f>
-        <v>46587</v>
+        <v>46636</v>
       </c>
       <c r="DC5" s="53">
         <f>DB5+7</f>
-        <v>46594</v>
+        <v>46643</v>
       </c>
       <c r="DD5" s="59" t="s">
         <v>40</v>
       </c>
       <c r="DE5" s="55">
         <f>DC5+7</f>
-        <v>46601</v>
+        <v>46650</v>
       </c>
       <c r="DF5" s="56">
         <f>DE5+7</f>
-        <v>46608</v>
+        <v>46657</v>
       </c>
       <c r="DG5" s="56">
         <f>DF5+7</f>
-        <v>46615</v>
+        <v>46664</v>
       </c>
       <c r="DH5" s="56">
         <f>DG5+7</f>
-        <v>46622</v>
+        <v>46671</v>
       </c>
       <c r="DI5" s="56">
         <f>DH5+7</f>
-        <v>46629</v>
+        <v>46678</v>
       </c>
       <c r="DJ5" s="53">
         <f>DI5+7</f>
-        <v>46636</v>
+        <v>46685</v>
       </c>
       <c r="DK5" s="59" t="s">
         <v>40</v>
       </c>
       <c r="DL5" s="55">
         <f>DJ5+7</f>
-        <v>46643</v>
+        <v>46692</v>
       </c>
       <c r="DM5" s="56">
         <f>DL5+7</f>
-        <v>46650</v>
+        <v>46699</v>
       </c>
       <c r="DN5" s="56">
         <f>DM5+7</f>
-        <v>46657</v>
+        <v>46706</v>
       </c>
       <c r="DO5" s="53">
         <f>DN5+7</f>
-        <v>46664</v>
+        <v>46713</v>
       </c>
       <c r="DP5" s="60" t="s">
         <v>41</v>
@@ -4132,417 +4131,416 @@
         <v>46005</v>
       </c>
       <c r="N6" s="63">
-        <f>N5+6</f>
-        <v>46012</v>
+        <v>46061</v>
       </c>
       <c r="O6" s="67" t="s">
         <v>45</v>
       </c>
       <c r="P6" s="65">
         <f>P5+6</f>
-        <v>46019</v>
+        <v>46068</v>
       </c>
       <c r="Q6" s="66">
         <f>Q5+6</f>
-        <v>46026</v>
+        <v>46075</v>
       </c>
       <c r="R6" s="66">
         <f>R5+6</f>
-        <v>46033</v>
+        <v>46082</v>
       </c>
       <c r="S6" s="66">
         <f>S5+6</f>
-        <v>46040</v>
+        <v>46089</v>
       </c>
       <c r="T6" s="66">
         <f>T5+6</f>
-        <v>46047</v>
+        <v>46096</v>
       </c>
       <c r="U6" s="66">
         <f>U5+6</f>
-        <v>46054</v>
+        <v>46103</v>
       </c>
       <c r="V6" s="66">
         <f>V5+6</f>
-        <v>46061</v>
+        <v>46110</v>
       </c>
       <c r="W6" s="66">
         <f>W5+6</f>
-        <v>46068</v>
+        <v>46117</v>
       </c>
       <c r="X6" s="66">
         <f>X5+6</f>
-        <v>46075</v>
+        <v>46124</v>
       </c>
       <c r="Y6" s="66">
         <f>Y5+6</f>
-        <v>46082</v>
+        <v>46131</v>
       </c>
       <c r="Z6" s="66">
         <f>Z5+6</f>
-        <v>46089</v>
+        <v>46138</v>
       </c>
       <c r="AA6" s="63">
         <f>AA5+6</f>
-        <v>46096</v>
+        <v>46145</v>
       </c>
       <c r="AB6" s="67" t="s">
         <v>45</v>
       </c>
       <c r="AC6" s="65">
         <f>AC5+6</f>
-        <v>46103</v>
+        <v>46152</v>
       </c>
       <c r="AD6" s="66">
         <f>AD5+6</f>
-        <v>46110</v>
+        <v>46159</v>
       </c>
       <c r="AE6" s="66">
         <f>AE5+6</f>
-        <v>46117</v>
+        <v>46166</v>
       </c>
       <c r="AF6" s="66">
         <f>AF5+6</f>
-        <v>46124</v>
+        <v>46173</v>
       </c>
       <c r="AG6" s="66">
         <f>AG5+6</f>
-        <v>46131</v>
+        <v>46180</v>
       </c>
       <c r="AH6" s="66">
         <f>AH5+6</f>
-        <v>46138</v>
+        <v>46187</v>
       </c>
       <c r="AI6" s="66">
         <f>AI5+6</f>
-        <v>46145</v>
+        <v>46194</v>
       </c>
       <c r="AJ6" s="66">
         <f>AJ5+6</f>
-        <v>46152</v>
+        <v>46201</v>
       </c>
       <c r="AK6" s="66">
         <f>AK5+6</f>
-        <v>46159</v>
+        <v>46208</v>
       </c>
       <c r="AL6" s="66">
         <f>AL5+6</f>
-        <v>46166</v>
+        <v>46215</v>
       </c>
       <c r="AM6" s="66">
         <f>AM5+6</f>
-        <v>46173</v>
+        <v>46222</v>
       </c>
       <c r="AN6" s="63">
         <f>AN5+6</f>
-        <v>46180</v>
+        <v>46229</v>
       </c>
       <c r="AO6" s="68" t="s">
         <v>46</v>
       </c>
       <c r="AP6" s="65">
         <f>AP5+6</f>
-        <v>46187</v>
+        <v>46236</v>
       </c>
       <c r="AQ6" s="66">
         <f>AQ5+6</f>
-        <v>46194</v>
+        <v>46243</v>
       </c>
       <c r="AR6" s="66">
         <f>AR5+6</f>
-        <v>46201</v>
+        <v>46250</v>
       </c>
       <c r="AS6" s="66">
         <f>AS5+6</f>
-        <v>46208</v>
+        <v>46257</v>
       </c>
       <c r="AT6" s="66">
         <f>AT5+6</f>
-        <v>46215</v>
+        <v>46264</v>
       </c>
       <c r="AU6" s="66">
         <f>AU5+6</f>
-        <v>46222</v>
+        <v>46271</v>
       </c>
       <c r="AV6" s="66">
         <f>AV5+6</f>
-        <v>46229</v>
+        <v>46278</v>
       </c>
       <c r="AW6" s="66">
         <f>AW5+6</f>
-        <v>46236</v>
+        <v>46285</v>
       </c>
       <c r="AX6" s="66">
         <f>AX5+6</f>
-        <v>46243</v>
+        <v>46292</v>
       </c>
       <c r="AY6" s="66">
         <f>AY5+6</f>
-        <v>46250</v>
+        <v>46299</v>
       </c>
       <c r="AZ6" s="66">
         <f>AZ5+6</f>
-        <v>46257</v>
+        <v>46306</v>
       </c>
       <c r="BA6" s="63">
         <f>BA5+6</f>
-        <v>46264</v>
+        <v>46313</v>
       </c>
       <c r="BB6" s="68" t="s">
         <v>46</v>
       </c>
       <c r="BC6" s="65">
         <f>BC5+6</f>
-        <v>46271</v>
+        <v>46320</v>
       </c>
       <c r="BD6" s="66">
         <f>BD5+6</f>
-        <v>46278</v>
+        <v>46327</v>
       </c>
       <c r="BE6" s="66">
         <f>BE5+6</f>
-        <v>46285</v>
+        <v>46334</v>
       </c>
       <c r="BF6" s="66">
         <f>BF5+6</f>
-        <v>46292</v>
+        <v>46341</v>
       </c>
       <c r="BG6" s="66">
         <f>BG5+6</f>
-        <v>46299</v>
+        <v>46348</v>
       </c>
       <c r="BH6" s="66">
         <f>BH5+6</f>
-        <v>46306</v>
+        <v>46355</v>
       </c>
       <c r="BI6" s="66">
         <f>BI5+6</f>
-        <v>46313</v>
+        <v>46362</v>
       </c>
       <c r="BJ6" s="66">
         <f>BJ5+6</f>
-        <v>46320</v>
+        <v>46369</v>
       </c>
       <c r="BK6" s="66">
         <f>BK5+6</f>
-        <v>46327</v>
+        <v>46376</v>
       </c>
       <c r="BL6" s="66">
         <f>BL5+6</f>
-        <v>46334</v>
+        <v>46383</v>
       </c>
       <c r="BM6" s="66">
         <f>BM5+6</f>
-        <v>46341</v>
+        <v>46390</v>
       </c>
       <c r="BN6" s="63">
         <f>BN5+6</f>
-        <v>46348</v>
+        <v>46397</v>
       </c>
       <c r="BO6" s="68" t="s">
         <v>46</v>
       </c>
       <c r="BP6" s="65">
         <f>BP5+6</f>
-        <v>46355</v>
+        <v>46404</v>
       </c>
       <c r="BQ6" s="66">
         <f>BQ5+6</f>
-        <v>46362</v>
+        <v>46411</v>
       </c>
       <c r="BR6" s="66">
         <f>BR5+6</f>
-        <v>46369</v>
+        <v>46418</v>
       </c>
       <c r="BS6" s="66">
         <f>BS5+6</f>
-        <v>46376</v>
+        <v>46425</v>
       </c>
       <c r="BT6" s="66">
         <f>BT5+6</f>
-        <v>46383</v>
+        <v>46432</v>
       </c>
       <c r="BU6" s="66">
         <f>BU5+6</f>
-        <v>46390</v>
+        <v>46439</v>
       </c>
       <c r="BV6" s="66">
         <f>BV5+6</f>
-        <v>46397</v>
+        <v>46446</v>
       </c>
       <c r="BW6" s="63">
         <f>BW5+6</f>
-        <v>46404</v>
+        <v>46453</v>
       </c>
       <c r="BX6" s="68" t="s">
         <v>46</v>
       </c>
       <c r="BY6" s="65">
         <f>BY5+6</f>
-        <v>46411</v>
+        <v>46460</v>
       </c>
       <c r="BZ6" s="66">
         <f>BZ5+6</f>
-        <v>46418</v>
+        <v>46467</v>
       </c>
       <c r="CA6" s="66">
         <f>CA5+6</f>
-        <v>46425</v>
+        <v>46474</v>
       </c>
       <c r="CB6" s="66">
         <f>CB5+6</f>
-        <v>46432</v>
+        <v>46481</v>
       </c>
       <c r="CC6" s="66">
         <f>CC5+6</f>
-        <v>46439</v>
+        <v>46488</v>
       </c>
       <c r="CD6" s="66">
         <f>CD5+6</f>
-        <v>46446</v>
+        <v>46495</v>
       </c>
       <c r="CE6" s="66">
         <f>CE5+6</f>
-        <v>46453</v>
+        <v>46502</v>
       </c>
       <c r="CF6" s="63">
         <f>CF5+6</f>
-        <v>46460</v>
+        <v>46509</v>
       </c>
       <c r="CG6" s="69" t="s">
         <v>47</v>
       </c>
       <c r="CH6" s="65">
         <f>CH5+6</f>
-        <v>46467</v>
+        <v>46516</v>
       </c>
       <c r="CI6" s="66">
         <f>CI5+6</f>
-        <v>46474</v>
+        <v>46523</v>
       </c>
       <c r="CJ6" s="66">
         <f>CJ5+6</f>
-        <v>46481</v>
+        <v>46530</v>
       </c>
       <c r="CK6" s="66">
         <f>CK5+6</f>
-        <v>46488</v>
+        <v>46537</v>
       </c>
       <c r="CL6" s="66">
         <f>CL5+6</f>
-        <v>46495</v>
+        <v>46544</v>
       </c>
       <c r="CM6" s="66">
         <f>CM5+6</f>
-        <v>46502</v>
+        <v>46551</v>
       </c>
       <c r="CN6" s="66">
         <f>CN5+6</f>
-        <v>46509</v>
+        <v>46558</v>
       </c>
       <c r="CO6" s="63">
         <f>CO5+6</f>
-        <v>46516</v>
+        <v>46565</v>
       </c>
       <c r="CP6" s="69" t="s">
         <v>47</v>
       </c>
       <c r="CQ6" s="65">
         <f>CQ5+6</f>
-        <v>46523</v>
+        <v>46572</v>
       </c>
       <c r="CR6" s="66">
         <f>CR5+6</f>
-        <v>46530</v>
+        <v>46579</v>
       </c>
       <c r="CS6" s="66">
         <f>CS5+6</f>
-        <v>46537</v>
+        <v>46586</v>
       </c>
       <c r="CT6" s="66">
         <f>CT5+6</f>
-        <v>46544</v>
+        <v>46593</v>
       </c>
       <c r="CU6" s="66">
         <f>CU5+6</f>
-        <v>46551</v>
+        <v>46600</v>
       </c>
       <c r="CV6" s="63">
         <f>CV5+6</f>
-        <v>46558</v>
+        <v>46607</v>
       </c>
       <c r="CW6" s="69" t="s">
         <v>47</v>
       </c>
       <c r="CX6" s="65">
         <f>CX5+6</f>
-        <v>46565</v>
+        <v>46614</v>
       </c>
       <c r="CY6" s="66">
         <f>CY5+6</f>
-        <v>46572</v>
+        <v>46621</v>
       </c>
       <c r="CZ6" s="66">
         <f>CZ5+6</f>
-        <v>46579</v>
+        <v>46628</v>
       </c>
       <c r="DA6" s="66">
         <f>DA5+6</f>
-        <v>46586</v>
+        <v>46635</v>
       </c>
       <c r="DB6" s="66">
         <f>DB5+6</f>
-        <v>46593</v>
+        <v>46642</v>
       </c>
       <c r="DC6" s="63">
         <f>DC5+6</f>
-        <v>46600</v>
+        <v>46649</v>
       </c>
       <c r="DD6" s="69" t="s">
         <v>47</v>
       </c>
       <c r="DE6" s="65">
         <f>DE5+6</f>
-        <v>46607</v>
+        <v>46656</v>
       </c>
       <c r="DF6" s="66">
         <f>DF5+6</f>
-        <v>46614</v>
+        <v>46663</v>
       </c>
       <c r="DG6" s="66">
         <f>DG5+6</f>
-        <v>46621</v>
+        <v>46670</v>
       </c>
       <c r="DH6" s="66">
         <f>DH5+6</f>
-        <v>46628</v>
+        <v>46677</v>
       </c>
       <c r="DI6" s="66">
         <f>DI5+6</f>
-        <v>46635</v>
+        <v>46684</v>
       </c>
       <c r="DJ6" s="63">
         <f>DJ5+6</f>
-        <v>46642</v>
+        <v>46691</v>
       </c>
       <c r="DK6" s="69" t="s">
         <v>47</v>
       </c>
       <c r="DL6" s="65">
         <f>DL5+6</f>
-        <v>46649</v>
+        <v>46698</v>
       </c>
       <c r="DM6" s="66">
         <f>DM5+6</f>
-        <v>46656</v>
+        <v>46705</v>
       </c>
       <c r="DN6" s="66">
         <f>DN5+6</f>
-        <v>46663</v>
+        <v>46712</v>
       </c>
       <c r="DO6" s="63">
         <f>DO5+6</f>
-        <v>46670</v>
+        <v>46719</v>
       </c>
       <c r="DP6" s="70" t="s">
         <v>48</v>

</xml_diff>